<commit_message>
Minor changes in Client BOM
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/Client_BOM_Bottom_Board.xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/Client_BOM_Bottom_Board.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25330"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CFDA366-B582-43DA-82D5-D3D67B89062A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="179">
   <si>
     <t>Component list</t>
   </si>
@@ -53,12 +52,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>SM_Bottom_Board.PrjPcb</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
     <t>Designator</t>
   </si>
   <si>
@@ -563,19 +556,22 @@
     <t>DFN1006P2E</t>
   </si>
   <si>
-    <t>Bill of Materials for Project (Smartmotors)</t>
-  </si>
-  <si>
-    <t>(Smartmotors)</t>
-  </si>
-  <si>
     <t>C2, C3, C4, C5, C6, C7, C8, C9, C10, C11, C15, C20, C32, C33, C34, C35, C36, C37, C50 , CF1</t>
+  </si>
+  <si>
+    <t>Bottom_Board</t>
+  </si>
+  <si>
+    <t>Smart Motors</t>
+  </si>
+  <si>
+    <t>Bill of Materials for Project Smart Motors</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -1145,6 +1141,21 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1153,21 +1164,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1212,7 +1208,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1508,7 +1504,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1534,9 +1530,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
     </row>
     <row r="2" spans="1:11" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1547,7 +1543,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="53" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -1564,13 +1560,13 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="54" t="s">
-        <v>7</v>
+        <v>176</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
-      <c r="K3" s="58"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1581,13 +1577,13 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="55" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
-      <c r="K4" s="59"/>
+      <c r="K4" s="64"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1597,14 +1593,12 @@
         <v>3</v>
       </c>
       <c r="E5" s="12"/>
-      <c r="F5" s="56" t="s">
-        <v>8</v>
-      </c>
+      <c r="F5" s="56"/>
       <c r="G5" s="14"/>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="59"/>
+      <c r="K5" s="64"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1617,7 +1611,7 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
-      <c r="K6" s="59"/>
+      <c r="K6" s="64"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1630,7 +1624,7 @@
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
-      <c r="K7" s="59"/>
+      <c r="K7" s="64"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1643,67 +1637,67 @@
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
-      <c r="K8" s="59"/>
+      <c r="K8" s="64"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="60" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="K9" s="31" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="62">
+      <c r="B10" s="59">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="60" t="s">
-        <v>163</v>
+      <c r="C10" s="57" t="s">
+        <v>161</v>
       </c>
       <c r="D10" s="41" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E10" s="38" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J10" s="37">
         <v>1</v>
@@ -1712,30 +1706,30 @@
     </row>
     <row r="11" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="62">
+      <c r="B11" s="59">
         <f t="shared" ref="B11:B40" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="61" t="s">
-        <v>163</v>
+      <c r="C11" s="58" t="s">
+        <v>161</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E11" s="40" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F11" s="39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H11" s="39" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I11" s="40" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J11" s="39">
         <v>20</v>
@@ -1744,30 +1738,30 @@
     </row>
     <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="62">
+      <c r="B12" s="59">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="64" t="s">
-        <v>163</v>
+      <c r="C12" s="61" t="s">
+        <v>161</v>
       </c>
       <c r="D12" s="41" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E12" s="38" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J12" s="37">
         <v>1</v>
@@ -1776,30 +1770,30 @@
     </row>
     <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="62">
+      <c r="B13" s="59">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="61" t="s">
-        <v>163</v>
+      <c r="C13" s="58" t="s">
+        <v>161</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E13" s="40" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H13" s="39" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I13" s="40" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J13" s="39">
         <v>2</v>
@@ -1808,30 +1802,30 @@
     </row>
     <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="62">
+      <c r="B14" s="59">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="64" t="s">
-        <v>163</v>
+      <c r="C14" s="61" t="s">
+        <v>161</v>
       </c>
       <c r="D14" s="41" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J14" s="37">
         <v>2</v>
@@ -1840,30 +1834,30 @@
     </row>
     <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="62">
+      <c r="B15" s="59">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="61" t="s">
-        <v>163</v>
+      <c r="C15" s="58" t="s">
+        <v>161</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E15" s="40" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F15" s="39" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I15" s="40" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="J15" s="39">
         <v>2</v>
@@ -1872,30 +1866,30 @@
     </row>
     <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="62">
+      <c r="B16" s="59">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="64" t="s">
-        <v>163</v>
+      <c r="C16" s="61" t="s">
+        <v>161</v>
       </c>
       <c r="D16" s="41" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G16" s="38" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H16" s="37" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I16" s="38" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="J16" s="37">
         <v>1</v>
@@ -1904,30 +1898,30 @@
     </row>
     <row r="17" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="62">
+      <c r="B17" s="59">
         <f>ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
-      <c r="C17" s="61" t="s">
-        <v>164</v>
+      <c r="C17" s="58" t="s">
+        <v>162</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E17" s="40" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F17" s="39" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G17" s="40" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I17" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J17" s="39">
         <v>2</v>
@@ -1936,30 +1930,30 @@
     </row>
     <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="62">
+      <c r="B18" s="59">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="64" t="s">
-        <v>164</v>
+      <c r="C18" s="61" t="s">
+        <v>162</v>
       </c>
       <c r="D18" s="41" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F18" s="37" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G18" s="38" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H18" s="37" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I18" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J18" s="37">
         <v>1</v>
@@ -1968,30 +1962,30 @@
     </row>
     <row r="19" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="62">
+      <c r="B19" s="59">
         <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="61" t="s">
-        <v>165</v>
+      <c r="C19" s="58" t="s">
+        <v>163</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E19" s="40" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F19" s="39" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G19" s="40" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H19" s="39" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I19" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J19" s="39">
         <v>4</v>
@@ -2000,30 +1994,30 @@
     </row>
     <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="62">
+      <c r="B20" s="59">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="64" t="s">
-        <v>166</v>
+      <c r="C20" s="61" t="s">
+        <v>164</v>
       </c>
       <c r="D20" s="41" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E20" s="38" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G20" s="38" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H20" s="37" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I20" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J20" s="37">
         <v>1</v>
@@ -2032,30 +2026,30 @@
     </row>
     <row r="21" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="62">
+      <c r="B21" s="59">
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="61" t="s">
-        <v>165</v>
+      <c r="C21" s="58" t="s">
+        <v>163</v>
       </c>
       <c r="D21" s="42" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E21" s="40" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F21" s="39" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G21" s="40" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H21" s="39" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I21" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J21" s="39">
         <v>1</v>
@@ -2064,30 +2058,30 @@
     </row>
     <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="62">
+      <c r="B22" s="59">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="64" t="s">
-        <v>167</v>
+      <c r="C22" s="61" t="s">
+        <v>165</v>
       </c>
       <c r="D22" s="41" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E22" s="38" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G22" s="38" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H22" s="37" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I22" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J22" s="37">
         <v>1</v>
@@ -2096,30 +2090,30 @@
     </row>
     <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
-      <c r="B23" s="62">
+      <c r="B23" s="59">
         <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="61" t="s">
-        <v>168</v>
+      <c r="C23" s="58" t="s">
+        <v>166</v>
       </c>
       <c r="D23" s="42" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E23" s="40" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F23" s="39" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G23" s="40" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H23" s="39" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I23" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J23" s="39">
         <v>1</v>
@@ -2128,30 +2122,30 @@
     </row>
     <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
-      <c r="B24" s="62">
+      <c r="B24" s="59">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="64" t="s">
-        <v>169</v>
+      <c r="C24" s="61" t="s">
+        <v>167</v>
       </c>
       <c r="D24" s="41" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E24" s="38" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F24" s="37" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G24" s="38" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H24" s="37" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I24" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J24" s="37">
         <v>2</v>
@@ -2160,30 +2154,30 @@
     </row>
     <row r="25" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
-      <c r="B25" s="62">
+      <c r="B25" s="59">
         <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
-      <c r="C25" s="61" t="s">
-        <v>170</v>
+      <c r="C25" s="58" t="s">
+        <v>168</v>
       </c>
       <c r="D25" s="42" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E25" s="40" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F25" s="39" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G25" s="40" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H25" s="39" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I25" s="40" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J25" s="39">
         <v>40</v>
@@ -2192,30 +2186,30 @@
     </row>
     <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="62">
+      <c r="B26" s="59">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="64" t="s">
-        <v>170</v>
+      <c r="C26" s="61" t="s">
+        <v>168</v>
       </c>
       <c r="D26" s="41" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E26" s="38" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F26" s="37" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G26" s="38" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H26" s="37" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I26" s="38" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J26" s="37">
         <v>7</v>
@@ -2224,30 +2218,30 @@
     </row>
     <row r="27" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
-      <c r="B27" s="62">
+      <c r="B27" s="59">
         <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="61" t="s">
-        <v>170</v>
+      <c r="C27" s="58" t="s">
+        <v>168</v>
       </c>
       <c r="D27" s="42" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F27" s="39" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G27" s="40" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H27" s="39" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I27" s="40" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J27" s="39">
         <v>1</v>
@@ -2256,30 +2250,30 @@
     </row>
     <row r="28" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
-      <c r="B28" s="62">
+      <c r="B28" s="59">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="64" t="s">
-        <v>170</v>
+      <c r="C28" s="61" t="s">
+        <v>168</v>
       </c>
       <c r="D28" s="41" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E28" s="38" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F28" s="37" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G28" s="38" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H28" s="37" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I28" s="38" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J28" s="37">
         <v>2</v>
@@ -2288,30 +2282,30 @@
     </row>
     <row r="29" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
-      <c r="B29" s="62">
+      <c r="B29" s="59">
         <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
-      <c r="C29" s="61" t="s">
-        <v>170</v>
+      <c r="C29" s="58" t="s">
+        <v>168</v>
       </c>
       <c r="D29" s="42" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F29" s="39" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G29" s="40" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H29" s="39" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I29" s="40" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J29" s="39">
         <v>1</v>
@@ -2320,30 +2314,30 @@
     </row>
     <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
-      <c r="B30" s="62">
+      <c r="B30" s="59">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="64" t="s">
-        <v>170</v>
+      <c r="C30" s="61" t="s">
+        <v>168</v>
       </c>
       <c r="D30" s="41" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E30" s="38" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F30" s="37" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G30" s="38" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H30" s="37" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I30" s="38" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J30" s="37">
         <v>2</v>
@@ -2352,30 +2346,30 @@
     </row>
     <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
-      <c r="B31" s="62">
+      <c r="B31" s="59">
         <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
-      <c r="C31" s="61" t="s">
-        <v>89</v>
+      <c r="C31" s="58" t="s">
+        <v>87</v>
       </c>
       <c r="D31" s="42" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F31" s="39" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G31" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H31" s="39" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="I31" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J31" s="39">
         <v>8</v>
@@ -2384,30 +2378,30 @@
     </row>
     <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
-      <c r="B32" s="62">
+      <c r="B32" s="59">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C32" s="64" t="s">
-        <v>171</v>
+      <c r="C32" s="61" t="s">
+        <v>169</v>
       </c>
       <c r="D32" s="41" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E32" s="38" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F32" s="37" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G32" s="38" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H32" s="37" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I32" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J32" s="37">
         <v>1</v>
@@ -2416,30 +2410,30 @@
     </row>
     <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
-      <c r="B33" s="62">
+      <c r="B33" s="59">
         <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
-      <c r="C33" s="61" t="s">
-        <v>172</v>
+      <c r="C33" s="58" t="s">
+        <v>170</v>
       </c>
       <c r="D33" s="42" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E33" s="40" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G33" s="40" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H33" s="39" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I33" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J33" s="39">
         <v>1</v>
@@ -2448,30 +2442,30 @@
     </row>
     <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
-      <c r="B34" s="62">
+      <c r="B34" s="59">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C34" s="64" t="s">
-        <v>172</v>
+      <c r="C34" s="61" t="s">
+        <v>170</v>
       </c>
       <c r="D34" s="41" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E34" s="38" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F34" s="37" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G34" s="38" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H34" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I34" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J34" s="37">
         <v>1</v>
@@ -2480,30 +2474,30 @@
     </row>
     <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
-      <c r="B35" s="62">
+      <c r="B35" s="59">
         <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
-      <c r="C35" s="61" t="s">
-        <v>172</v>
+      <c r="C35" s="58" t="s">
+        <v>170</v>
       </c>
       <c r="D35" s="42" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E35" s="40" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F35" s="39" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G35" s="40" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H35" s="39" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I35" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J35" s="39">
         <v>1</v>
@@ -2512,30 +2506,30 @@
     </row>
     <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
-      <c r="B36" s="62">
+      <c r="B36" s="59">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C36" s="64" t="s">
-        <v>172</v>
+      <c r="C36" s="61" t="s">
+        <v>170</v>
       </c>
       <c r="D36" s="41" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E36" s="38" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F36" s="37" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G36" s="38" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H36" s="37" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I36" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J36" s="37">
         <v>1</v>
@@ -2544,30 +2538,30 @@
     </row>
     <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
-      <c r="B37" s="62">
+      <c r="B37" s="59">
         <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
-      <c r="C37" s="61" t="s">
-        <v>172</v>
+      <c r="C37" s="58" t="s">
+        <v>170</v>
       </c>
       <c r="D37" s="42" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E37" s="40" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F37" s="39" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G37" s="40" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H37" s="39" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I37" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J37" s="39">
         <v>1</v>
@@ -2576,30 +2570,30 @@
     </row>
     <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
-      <c r="B38" s="62">
+      <c r="B38" s="59">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="64" t="s">
-        <v>172</v>
+      <c r="C38" s="61" t="s">
+        <v>170</v>
       </c>
       <c r="D38" s="41" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E38" s="38" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F38" s="37" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G38" s="38" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H38" s="37" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I38" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J38" s="37">
         <v>1</v>
@@ -2608,30 +2602,30 @@
     </row>
     <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
-      <c r="B39" s="62">
+      <c r="B39" s="59">
         <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
-      <c r="C39" s="61" t="s">
-        <v>172</v>
+      <c r="C39" s="58" t="s">
+        <v>170</v>
       </c>
       <c r="D39" s="42" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E39" s="40" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F39" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G39" s="40" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H39" s="39" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I39" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J39" s="39">
         <v>1</v>
@@ -2640,30 +2634,30 @@
     </row>
     <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="62">
+      <c r="B40" s="59">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C40" s="64" t="s">
-        <v>173</v>
+      <c r="C40" s="61" t="s">
+        <v>171</v>
       </c>
       <c r="D40" s="41" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E40" s="38" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F40" s="37" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G40" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H40" s="37" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I40" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J40" s="37">
         <v>1</v>
@@ -2672,30 +2666,30 @@
     </row>
     <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="62">
+      <c r="B41" s="59">
         <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
-      <c r="C41" s="61" t="s">
-        <v>173</v>
+      <c r="C41" s="58" t="s">
+        <v>171</v>
       </c>
       <c r="D41" s="42" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E41" s="40" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F41" s="39" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G41" s="40" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H41" s="39" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I41" s="40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J41" s="39">
         <v>1</v>

</xml_diff>